<commit_message>
Momentum scan results 2026-08-21
</commit_message>
<xml_diff>
--- a/results/momentum_merged_2026-08-21.xlsx
+++ b/results/momentum_merged_2026-08-21.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D113"/>
+  <dimension ref="A1:D125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,12 +441,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ABOS</t>
+          <t>ABUS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ACIU</t>
+          <t>AACG</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -456,574 +456,574 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ARBE</t>
+          <t>AD</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ACCL</t>
+          <t>ASPCU</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ADIL</t>
+          <t>ABNB</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AD</t>
+          <t>HOWL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ARQ</t>
+          <t>AEC</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ACOG</t>
+          <t>ASST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>ABOS</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMOD</t>
+          <t>ICG</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>BGIN</t>
+          <t>ATLX</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ADUR</t>
+          <t>BRNX</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AEHR</t>
+          <t>ABXL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ASST</t>
+          <t>BHFAL</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>BTOC</t>
+          <t>CBAT</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>ACCL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AEI</t>
+          <t>BLNK</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BEEM</t>
+          <t>CEPO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CECO</t>
+          <t>ACFN</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AEHL</t>
+          <t>BORR</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AIFA</t>
+          <t>CFFI</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BHFAL</t>
+          <t>ACIU</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CELZ</t>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>CYPH</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AIIR</t>
+          <t>ACOG</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BLSH</t>
+          <t>CDLX</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CENN</t>
+          <t>CZFS</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ALVO</t>
+          <t>ACT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ALOT</t>
+          <t>CDTG</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BTCS</t>
+          <t>DMAA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CRGO</t>
+          <t>ADAG</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AMCX</t>
+          <t>CENN</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ALXO</t>
+          <t>ELMT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BTGO</t>
+          <t>ADAMH</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CTOR</t>
+          <t>CNTY</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AMLX</t>
+          <t>FUTU</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>AMPL</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CDTG</t>
+          <t>CPHC</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ELLA</t>
+          <t>GECCI</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>CRGO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DFDV</t>
+          <t>GIBO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FCFS</t>
+          <t>ADUR</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ARCT</t>
+          <t>DEFT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ANGX</t>
+          <t>HFBL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>EEIQ</t>
+          <t>ADUS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>GLE</t>
+          <t>DETX</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ATAI</t>
+          <t>HOLO</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>APGE</t>
+          <t>AEHL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ELVR</t>
+          <t>DXST</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>GNSS</t>
+          <t>JATT</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>AIFA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>APLM</t>
+          <t>ELVR</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>EXOZ</t>
+          <t>JUNS</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>HAO</t>
+          <t>ALKT</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AUGO</t>
+          <t>EVAX</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>APPF</t>
+          <t>MSLE</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GOLD</t>
+          <t>ALM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>IXHL</t>
+          <t>EXOZ</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AVTR</t>
+          <t>NAKA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ALVO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>HOLO</t>
+          <t>FABC</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>NTRB</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AXGN</t>
+          <t>AMCR</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AREC</t>
+          <t>FKWL</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ICG</t>
+          <t>OXLCI</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>JVA</t>
+          <t>AMCX</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>GMTL</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ARGX</t>
+          <t>PBHC</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>IRD</t>
+          <t>AMLX</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>KXIN</t>
+          <t>HAO</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BAFN</t>
+          <t>PCAP</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ARTNA</t>
+          <t>AMR</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>KBSX</t>
+          <t>HTZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LUNR</t>
+          <t>TRON</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BLFS</t>
+          <t>AMTX</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ARTW</t>
+          <t>INKT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>KWY</t>
+          <t>ANGX</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MLGO</t>
+          <t>JSM</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>APGE</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ARX</t>
+          <t>JVA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LEE</t>
+          <t>APLM</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>MRAM</t>
+          <t>JYD</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BMNR</t>
+          <t>APPF</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ASBP</t>
+          <t>LNZA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LKQ</t>
+          <t>AQB</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MRM</t>
+          <t>MLGO</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BOSC</t>
+          <t>AQST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ATKR</t>
+          <t>OCG</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>NEGG</t>
+          <t>PAHC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>BRNX</t>
+          <t>ARCC</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AVBC</t>
+          <t>PPBT</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MSAI</t>
+          <t>ARCT</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>NWGL</t>
+          <t>PPIH</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BRR</t>
+          <t>ARGX</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>PTN</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>NAKA</t>
+          <t>ARTNA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>OPTX</t>
+          <t>QNTM</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BRZE</t>
+          <t>ASBP</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AWR</t>
+          <t>SEV</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ORBS</t>
+          <t>ASMB</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>REA</t>
+          <t>SJ</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BULL</t>
+          <t>ATAI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>AXTI</t>
+          <t>SLDP</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PHIO</t>
+          <t>ATKR</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1035,320 +1035,320 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CABA</t>
+          <t>ATRC</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>SWVL</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PPIH</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SRZN</t>
+          <t>TMUS</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAI</t>
+          <t>AUGO</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BCSS</t>
+          <t>WSE</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PRTS</t>
+          <t>AURA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>VIVO</t>
+          <t>AUTL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CARL</t>
+          <t>AVAH</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BEEP</t>
+          <t>AVO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PUSA</t>
+          <t>AVR</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>AVTR</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BFRI</t>
+          <t>AXIN</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SEV</t>
+          <t>AYTU</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>CDLR</t>
+          <t>BANX</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>BGDE</t>
+          <t>BBIO</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SHAZ</t>
+          <t>BCTX</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CETY</t>
+          <t>BDTX</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>BIOX</t>
+          <t>BEEM</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>SPCB</t>
+          <t>BEEP</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CFFI</t>
+          <t>BETA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>BGDE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>BIOX</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
           <t>BIXI</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>STEX</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>CGC</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BPYPP</t>
+          <t>BLKB</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SWVL</t>
+          <t>BLMN</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CGEN</t>
+          <t>BLSH</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>BMNR</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>BNTC</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CHSCO</t>
+          <t>BNTX</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>BRLT</t>
+          <t>BOLD</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>TRON</t>
+          <t>BPRN</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CJMB</t>
+          <t>BPYPO</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>BSBK</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>USAU</t>
+          <t>BRCB</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CLIR</t>
+          <t>BRR</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>BTU</t>
+          <t>BRZE</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CLLS</t>
+          <t>BSY</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>BUUU</t>
+          <t>BTCS</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>COCP</t>
+          <t>BTGO</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>BTU</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>COHU</t>
+          <t>BUDA</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>BYND</t>
+          <t>BULL</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>BULLW</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>BUUU</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CSTE</t>
+          <t>BVC</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>BWIN</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>CYPH</t>
+          <t>BYND</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CCEC</t>
+          <t>CABA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>CAI</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CDIO</t>
+          <t>CARL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>DMLP</t>
+          <t>CCC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>CCEC</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>DTIL</t>
+          <t>CCG</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CELH</t>
+          <t>CDLR</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>DWTX</t>
+          <t>CEG</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>CELH</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ELVN</t>
+          <t>CELU</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1358,1537 +1358,1809 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ENTX</t>
+          <t>CGC</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>CGEN</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>CHCI</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>EXE</t>
-        </is>
-      </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>CHNR</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>CHTRP</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CHNR</t>
+          <t>CING</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>FBLG</t>
+          <t>CLMT</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CLYM</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>FRHC</t>
+          <t>CMCSA</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CHTRP</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>FUTU</t>
+          <t>CMTV</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CHYM</t>
+          <t>CNET</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>FWDI</t>
+          <t>CNR</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CING</t>
+          <t>COCP</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>GASS</t>
+          <t>CORT</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CLYM</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>CPBI</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CNOBP</t>
+          <t>CPRT</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>GLNG</t>
+          <t>CRSP</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CNR</t>
+          <t>CRVL</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>GNLN</t>
+          <t>CSAI</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CNSP</t>
+          <t>CSHR</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GOODO</t>
+          <t>CSTE</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>COCH</t>
+          <t>CSTL</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>GSHD</t>
+          <t>CSWC</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>COYA</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>HBIO</t>
+          <t>CTRM</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CPBI</t>
+          <t>CTSH</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>HFBL</t>
+          <t>CYCN</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CPRT</t>
+          <t>DAAQ</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>HMR</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CRBP</t>
+          <t>DBX</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>HQI</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CSAI</t>
+          <t>DDI</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>DERM</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CSWC</t>
+          <t>DFDV</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>DMLP</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CURI</t>
+          <t>DNMX</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>DNUT</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>DOX</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>IDYA</t>
+          <t>DRTS</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>DRUG</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>IMMR</t>
+          <t>DSGR</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>DHCNI</t>
+          <t>DTIL</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>IMPP</t>
+          <t>DWTX</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>DIBS</t>
+          <t>DXCM</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>EDRY</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>DJCO</t>
+          <t>EEIQ</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>IOVA</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>DMC</t>
+          <t>EFSI</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JATT</t>
+          <t>EGHA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>DOCU</t>
+          <t>ELBM</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>JCSE</t>
+          <t>ELVN</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>DOX</t>
+          <t>ENTX</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>LEXX</t>
+          <t>EROK</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>DRMA</t>
+          <t>ETON</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>MAKO</t>
+          <t>EXFY</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DSGR</t>
+          <t>EXLS</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>DTI</t>
+          <t>FBLG</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>MASS</t>
+          <t>FBRX</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>DUOL</t>
+          <t>FCUV</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>FEAM</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>DXCM</t>
+          <t>FHTX</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>FIGR</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>EDRY</t>
+          <t>FIVE</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MESO</t>
+          <t>FIZZ</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>FLNT</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>MICC</t>
+          <t>FLXS</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>EGHA</t>
+          <t>FLYW</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>FNKO</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>FOX</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>FOXF</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>EMBC</t>
+          <t>FRHC</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MSLE</t>
+          <t>FRNM</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>EROK</t>
+          <t>FVAV</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>FVN</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ETON</t>
+          <t>FWDI</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>NDSN</t>
+          <t>FWONA</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>EXFY</t>
+          <t>GAINZ</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>NEPH</t>
+          <t>GASS</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>GBDC</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>NHP</t>
+          <t>GCL</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>FCUV</t>
+          <t>GDYN</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>NKLR</t>
+          <t>GECC</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>FNKO</t>
+          <t>GECCG</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>GLBS</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>FRD</t>
+          <t>GLNG</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>NTRB</t>
+          <t>GOLD</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>FVAV</t>
+          <t>GOODO</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>NVCT</t>
+          <t>GP</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>FVN</t>
+          <t>GRDX</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>OGC</t>
+          <t>GROW</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>GAINZ</t>
+          <t>GRRR</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ONBPO</t>
+          <t>GRVY</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>GBDC</t>
+          <t>GSHD</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>OTLY</t>
+          <t>GTEC</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>GCBC</t>
+          <t>GTIM</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>OXLCI</t>
+          <t>GTM</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>GCL</t>
+          <t>GYRE</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>OXLCO</t>
+          <t>HAIN</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>GECC</t>
+          <t>HALO</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>GLAD</t>
+          <t>HELP</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>PANL</t>
+          <t>HLNE</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>GP</t>
+          <t>HMR</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>HNNA</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>GRDX</t>
+          <t>HNVR</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>PBAM</t>
+          <t>HQWWW</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>GRRR</t>
+          <t>HRZN</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PBHC</t>
+          <t>HTFL</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>GTEC</t>
+          <t>HURC</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>PCAP</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>GTIM</t>
+          <t>HYPD</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PCYO</t>
+          <t>IBKR</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>ICLR</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>PFX</t>
+          <t>IDYA</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>HBANL</t>
+          <t>IMMX</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PGEN</t>
+          <t>IMPP</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>HCM</t>
+          <t>IMRX</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>PMVP</t>
+          <t>IMUX</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>HELP</t>
+          <t>INBKZ</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PRLD</t>
+          <t>INBX</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>HMH</t>
+          <t>INCY</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>PRPO</t>
+          <t>INDI</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>HPK</t>
+          <t>INFQ</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PRQR</t>
+          <t>INMB</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>HTFL</t>
+          <t>INO</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>PRZO</t>
+          <t>INTU</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>HTO</t>
+          <t>IPHA</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PSNL</t>
+          <t>IRD</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>HUDI</t>
+          <t>JAN</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>PTGX</t>
+          <t>JANX</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>HWCPZ</t>
+          <t>JCSE</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PXS</t>
+          <t>JKHY</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>IBKR</t>
+          <t>JRSH</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>KELYA</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>KIDZ</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>QURE</t>
+          <t>KLTR</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>IFRX</t>
+          <t>KMDA</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>RDZN</t>
+          <t>KOPN</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>IMXI</t>
+          <t>KOYN</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>KPRX</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>INBKZ</t>
+          <t>KROS</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>RILYN</t>
+          <t>KSPI</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>IPHA</t>
+          <t>KWY</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>RMTI</t>
+          <t>KZIA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>IVDA</t>
+          <t>LAUR</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>LEGH</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>JAN</t>
+          <t>LEXX</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SATA</t>
+          <t>LGVN</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>JRSH</t>
+          <t>LIFE</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>SBET</t>
+          <t>LKQ</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>JUNS</t>
+          <t>LKSP</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SCZM</t>
+          <t>LPBB</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>KELYA</t>
+          <t>LYEL</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>SEIC</t>
+          <t>LYFT</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>KIDZ</t>
+          <t>MACI</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SELF</t>
+          <t>MBINL</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>KLTR</t>
+          <t>MBUU</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>MCGA</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>KOYN</t>
+          <t>MDLZ</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SMJF</t>
+          <t>MEDP</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>KPRX</t>
+          <t>MELI</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>SOPH</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>KSPI</t>
+          <t>MFIN</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SRTA</t>
+          <t>MICC</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>KZIA</t>
+          <t>MINE</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>SSRM</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>LARK</t>
+          <t>MLAA</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>STKH</t>
+          <t>MLAB</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>LEGH</t>
+          <t>MMED</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>STRD</t>
+          <t>MMYT</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>LGVN</t>
+          <t>MOLN</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>STRK</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>MRX</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>TLIH</t>
+          <t>MYSE</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>LKSP</t>
+          <t>NAVI</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TLX</t>
+          <t>NBP</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>LPBB</t>
+          <t>NCI</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>TOP</t>
+          <t>NCT</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>LPSN</t>
+          <t>NDAQ</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TORO</t>
+          <t>NEGG</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>MACI</t>
+          <t>NEO</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>TRLV</t>
+          <t>NICM</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>MBINL</t>
+          <t>NIPG</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>NIQ</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>MCFT</t>
+          <t>NMFCZ</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>YDES</t>
+          <t>NPT</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>MCGA</t>
+          <t>NRC</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MDXH</t>
+          <t>NTHI</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>METCI</t>
+          <t>NTNX</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>MF</t>
+          <t>NTRA</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MFIN</t>
+          <t>NVAX</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>MGRT</t>
+          <t>NVCT</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>MINE</t>
+          <t>NWS</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>MLAA</t>
+          <t>NWSA</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>NWTG</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MRDN</t>
+          <t>NXPL</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>MSGY</t>
+          <t>OABI</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>OBIO</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>NCT</t>
+          <t>ODTX</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>NEOV</t>
+          <t>OESX</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>NHPBP</t>
+          <t>OGC</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>NICM</t>
+          <t>OGG</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>NMFCZ</t>
+          <t>OMER</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>NTHI</t>
+          <t>OMEX</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>NUAI</t>
+          <t>ONC</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>OPRT</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>ORBS</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>OXLCM</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>NWTG</t>
+          <t>PAA</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>NXPL</t>
+          <t>PAGP</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>OABI</t>
+          <t>PANL</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>OCSL</t>
+          <t>PAX</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>ODTX</t>
+          <t>PAYS</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>OGG</t>
+          <t>PAYX</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>OMER</t>
+          <t>PBAM</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>OMEX</t>
+          <t>PCTY</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>ORKA</t>
+          <t>PCVX</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>OXLCM</t>
+          <t>PEP</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>OXLCZ</t>
+          <t>PEPG</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>PFSA</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>PAYS</t>
+          <t>PFX</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>PCTY</t>
+          <t>PHVS</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PHOE</t>
+          <t>PLSE</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PHVS</t>
+          <t>PMN</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>PLPC</t>
+          <t>PMVP</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>PLRX</t>
+          <t>PNRG</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PLSE</t>
+          <t>PPC</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PMTW</t>
+          <t>PRAA</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>PNRG</t>
+          <t>PRAX</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>PRAX</t>
+          <t>PRLD</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>PROV</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PRHI</t>
+          <t>PRQR</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
+          <t>PRZO</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
           <t>PS</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>PTC</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
+          <t>PSNL</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
           <t>PTEN</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>PXLW</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>PYPD</t>
-        </is>
-      </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>RCBC</t>
+          <t>PURR</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>RDNT</t>
+          <t>PXLW</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>RDVT</t>
+          <t>PXS</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>RGLD</t>
+          <t>PYPD</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>RMNI</t>
+          <t>PYPL</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>RNXT</t>
+          <t>QQQX</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>QURE</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>RRGB</t>
+          <t>RCBC</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>RUM</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>RWAYI</t>
+          <t>RCMT</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>SAIH</t>
+          <t>RDZN</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>SBMT</t>
+          <t>REAX</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>SCYX</t>
+          <t>REFI</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>SEGG</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>SENEA</t>
+          <t>RENT</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>SFBC</t>
+          <t>RGLD</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>SHC</t>
+          <t>RILYG</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SIEB</t>
+          <t>RMBI</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>RMCO</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>SLMBP</t>
+          <t>RMNI</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>SLP</t>
+          <t>RNAC</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>ROIV</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>SWKHL</t>
+          <t>ROKU</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>RUM</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>RVMD</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>THH</t>
+          <t>RWAYI</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>TLF</t>
+          <t>RXRX</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>TPCS</t>
+          <t>SAFT</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>TRIN</t>
+          <t>SAIH</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>TRMD</t>
+          <t>SATA</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>VACI</t>
+          <t>SBET</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>VCTR</t>
+          <t>SBLK</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>VERU</t>
+          <t>SBMT</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>VOXR</t>
+          <t>SCWO</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>VSECU</t>
+          <t>SCYX</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>WSBCO</t>
+          <t>SDGR</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>WSTN</t>
+          <t>SEIC</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>YORW</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr"/>
-      <c r="C113" t="inlineStr"/>
-      <c r="D113" t="inlineStr"/>
+          <t>SHIP</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>SIBN</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>SLDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>SLMBP</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>SLNG</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>SLP</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>SOPH</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>SPCB</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>SPT</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>SPTX</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>SQFTP</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>SRTA</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>SSRM</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>STEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>STRC</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>STRD</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>STRF</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>STRK</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>TAYD</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>TECX</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>THH</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>TILE</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>TIPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>TLF</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>TOP</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>TORO</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>TRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>TRLV</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>TRMB</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>TRMD</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>VERU</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>VGNT</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>VMET</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>VOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>VOXR</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>VSECU</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>WSBCO</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>WSTN</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>XXI</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>ZSTK</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>